<commit_message>
Update data package at: 2025-09-30T12:55:34Z
</commit_message>
<xml_diff>
--- a/data-raw/base_qdd_fiscal_fonte_95_2025.xlsx
+++ b/data-raw/base_qdd_fiscal_fonte_95_2025.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\splor-mg\dados-qdd-fonte-95\data-raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\splor-mg\code\dados-qdd-fonte-95\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89C9D767-23C6-4343-A7AB-E0AD00467901}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4995" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-4995" yWindow="-16320" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="base_qdd_fiscal" sheetId="1" r:id="rId1"/>
@@ -18,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">base_qdd_fiscal!$A$1:$AE$39</definedName>
   </definedNames>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -407,7 +406,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -748,7 +747,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AE39"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4463,7 +4462,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AE39" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:AE39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>